<commit_message>
update g3 stocks, scar stocks, move weight from g3 lowers
</commit_message>
<xml_diff>
--- a/changes/g3-stocks.xlsx
+++ b/changes/g3-stocks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yifan/Documents/deadline-balancing/changes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6348387-E74D-4265-A4DE-68B500FA95B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1F2115-9CD9-A943-8CA8-52D37C146DDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="m4-barrels" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
   <si>
     <t>new</t>
   </si>
@@ -44,112 +44,127 @@
     <t>pretty_name</t>
   </si>
   <si>
+    <t>ergonomics</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>horizontal_recoil</t>
+  </si>
+  <si>
+    <t>vertical_recoil</t>
+  </si>
+  <si>
+    <t>magazine_capacity</t>
+  </si>
+  <si>
+    <t>barrel_deviation</t>
+  </si>
+  <si>
+    <t>bullet_damage</t>
+  </si>
+  <si>
+    <t>bullet_velocity</t>
+  </si>
+  <si>
+    <t>buck_barrel_deviation</t>
+  </si>
+  <si>
+    <t>fire_rate</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
     <t>strength</t>
   </si>
   <si>
-    <t>ergonomics</t>
-  </si>
-  <si>
-    <t>weight</t>
-  </si>
-  <si>
-    <t>horizontal_recoil</t>
-  </si>
-  <si>
-    <t>vertical_recoil</t>
-  </si>
-  <si>
-    <t>magazine_capacity</t>
-  </si>
-  <si>
-    <t>bullet_damage</t>
-  </si>
-  <si>
-    <t>bullet_velocity</t>
-  </si>
-  <si>
-    <t>fire_rate</t>
-  </si>
-  <si>
-    <t>price</t>
-  </si>
-  <si>
-    <t>barrel_deviation</t>
-  </si>
-  <si>
-    <t>buck_barrel_deviation</t>
-  </si>
-  <si>
     <t>hk_g3_endplate</t>
   </si>
   <si>
-    <t>HK G3 Endplate</t>
+    <t>KG-31 Endplate</t>
   </si>
   <si>
     <t>hk_g3a3_stock_endplate</t>
   </si>
   <si>
-    <t>HK G3A3 Stock Endplate</t>
+    <t>KG-31a3 Stock Endplate</t>
   </si>
   <si>
     <t>hk_g3a3_stock_extendable_part</t>
   </si>
   <si>
-    <t>HK G3A3 Stock Extendable Part</t>
+    <t>KG-31a3 Stock Extendable Part</t>
   </si>
   <si>
     <t>hk_g3_std_fixed_plastic_stock</t>
   </si>
   <si>
-    <t>HK G3 Standard Fixed Plastic</t>
+    <t>KG-31 Standard Fixed Plastic</t>
+  </si>
+  <si>
+    <t>some guy said 12.5 oz without backplate</t>
   </si>
   <si>
     <t>haga_defense_hk_g3_acr_stock_adapter</t>
   </si>
   <si>
-    <t>Haga Defense HK G3 ACR Stock Adaptor</t>
+    <t>HAGA Defense KG-31 ACR</t>
   </si>
   <si>
     <t>ptr_hk_g3_milspec_ar15_buffer_tube_adapter</t>
   </si>
   <si>
-    <t>PTR HK G3 MilSpec AR15 Buffer Tube Adaptor</t>
+    <t>CTR KG-31 Milspec AR-15 Buffer Tube</t>
   </si>
   <si>
     <t>spuhr_g3_r410_stock_assembly_adapter</t>
   </si>
   <si>
-    <t>Spuhr G3 R410 Stock Assembly Adaptor</t>
+    <t>Spuhr KG-31 R-410 Stock Assembly</t>
   </si>
   <si>
     <t>hk_psg1_stock_buttpad</t>
   </si>
   <si>
-    <t>HK PSG-1 Stock Buttpad</t>
+    <t>SKG-31 Stock</t>
   </si>
   <si>
     <t>hk_psg1_stock_cheek_rest</t>
   </si>
   <si>
-    <t>HK PSG-1 Stock Cheek Rest</t>
-  </si>
-  <si>
     <t>hk_psg1_stock_base</t>
   </si>
   <si>
-    <t>HK Sniper PSG-1 Version 2 Stock Assembly</t>
+    <t>Sniper SKG-31 Version 2</t>
   </si>
   <si>
     <t>spuhr_g3_r410_stock_assembly_stock</t>
   </si>
   <si>
-    <t>Spuhr G3 R410 Stock</t>
+    <t>Spuhr KG-31 R-410</t>
   </si>
   <si>
     <t>spuhr_g3_r410_stock_assembly_cheek_pad</t>
   </si>
   <si>
-    <t>Spuhr G3 R410 Stock Cheek Pad</t>
+    <t>dynamic_development_group_sas_acr_stock_retractor</t>
+  </si>
+  <si>
+    <t>Dynamic Development Group SAS Adaptive ACR Retractor</t>
+  </si>
+  <si>
+    <t>dynamic_development_group_sas_acr_stock_cheek_pad</t>
+  </si>
+  <si>
+    <t>Dynamic Development Group SAS Adaptive ACR Stock</t>
+  </si>
+  <si>
+    <t>dynamic_development_group_sas_acr_stock</t>
+  </si>
+  <si>
+    <t>MOE Carbine</t>
   </si>
   <si>
     <t>default</t>
@@ -161,168 +176,23 @@
     <t>acr</t>
   </si>
   <si>
-    <t>dynamic_development_group_sas_acr_stock</t>
-  </si>
-  <si>
-    <t>Kinetic Development Group SAS Adaptive ACR Stock</t>
-  </si>
-  <si>
-    <t>dynamic_development_group_sas_acr_stock_cheek_pad</t>
-  </si>
-  <si>
-    <t>dynamic_development_group_sas_acr_stock_retractor</t>
-  </si>
-  <si>
-    <t>Kinetic Development Group SAS Adaptive ACR Retractor</t>
-  </si>
-  <si>
     <t>psg1</t>
   </si>
   <si>
-    <t>MOE Carbine</t>
+    <t>spuhr</t>
   </si>
   <si>
     <t>buffer</t>
-  </si>
-  <si>
-    <t>spuhr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -335,188 +205,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -524,205 +221,16 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1034,19 +542,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N39"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P39"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="42.140625" customWidth="1"/>
-    <col min="3" max="22" width="6.7109375" customWidth="1"/>
+    <col min="1" max="1" width="31.1640625" customWidth="1"/>
+    <col min="2" max="2" width="42.1640625" customWidth="1"/>
+    <col min="3" max="22" width="6.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1054,22 +563,22 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>8</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
       </c>
       <c r="I2" t="s">
         <v>9</v>
@@ -1078,19 +587,19 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" t="s">
         <v>14</v>
       </c>
-      <c r="L2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1101,7 +610,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -1115,11 +624,11 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f>C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*10+J3/300</f>
-        <v>-1.6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" ref="N3:N39" si="0">C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*10+J3/300</f>
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1130,7 +639,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="1">
-        <v>0.1</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -1144,11 +653,11 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <f t="shared" ref="N4:N36" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*5+I4*10+J4/300</f>
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-2.8000000000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1156,26 +665,26 @@
         <v>20</v>
       </c>
       <c r="C5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E5">
         <v>-7</v>
       </c>
       <c r="F5">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="M5">
         <v>0</v>
       </c>
       <c r="N5">
         <f t="shared" si="0"/>
-        <v>21.6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>22.200000000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1183,10 +692,10 @@
         <v>22</v>
       </c>
       <c r="C6">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D6">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="E6">
         <v>-12</v>
@@ -1199,72 +708,72 @@
       </c>
       <c r="N6">
         <f t="shared" si="0"/>
-        <v>20.6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>21.8</v>
+      </c>
+      <c r="P6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E7">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M7">
         <v>1000</v>
       </c>
       <c r="N7">
         <f t="shared" si="0"/>
-        <v>1.2000000000000002</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="D8">
-        <v>7.0000000000000007E-2</v>
+        <v>0.06</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8">
-        <v>1</v>
-      </c>
-      <c r="H8">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="M8">
         <v>1200</v>
       </c>
       <c r="N8">
         <f t="shared" si="0"/>
-        <v>-4.3000000000000007</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9">
         <v>-2</v>
@@ -1286,12 +795,12 @@
         <v>-3.8</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -1307,12 +816,12 @@
         <v>0.59999999999999987</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
         <v>31</v>
-      </c>
-      <c r="B11" t="s">
-        <v>32</v>
       </c>
       <c r="C11">
         <v>4</v>
@@ -1328,7 +837,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -1336,10 +845,10 @@
         <v>34</v>
       </c>
       <c r="C12">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D12">
-        <v>0.26</v>
+        <v>0.35</v>
       </c>
       <c r="E12">
         <v>-4</v>
@@ -1355,10 +864,10 @@
       </c>
       <c r="N12">
         <f t="shared" si="0"/>
-        <v>16.850000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+        <v>14.049999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -1366,31 +875,31 @@
         <v>36</v>
       </c>
       <c r="C13">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D13">
-        <v>0.18</v>
+        <v>0.25</v>
       </c>
       <c r="E13">
         <v>-10</v>
       </c>
       <c r="F13">
-        <v>-18</v>
+        <v>-15</v>
       </c>
       <c r="M13">
         <v>0</v>
       </c>
       <c r="N13">
         <f t="shared" si="0"/>
-        <v>23.2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>37</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -1405,13 +914,16 @@
         <f t="shared" si="0"/>
         <v>1.2</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P14">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1423,16 +935,16 @@
         <v>0</v>
       </c>
       <c r="N15">
-        <f>C15-D15*20-E15*0.8-F15*0.6-H15*5+I15*10+J15/300</f>
+        <f t="shared" si="0"/>
         <v>-2.2000000000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C16">
         <v>4</v>
@@ -1444,47 +956,47 @@
         <v>0</v>
       </c>
       <c r="N16">
-        <f>C16-D16*20-E16*0.8-F16*0.6-H16*5+I16*10+J16/300</f>
+        <f t="shared" si="0"/>
         <v>3.2</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C17">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D17">
         <v>0.16</v>
       </c>
       <c r="E17">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="F17">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="M17">
         <v>1000</v>
       </c>
       <c r="N17">
-        <f>C17-D17*20-E17*0.8-F17*0.6-H17*5+I17*10+J17/300</f>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>21.400000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C18" s="1">
         <v>17</v>
       </c>
       <c r="D18" s="1">
-        <v>0.35000000000000003</v>
+        <v>0.37</v>
       </c>
       <c r="E18" s="1">
         <v>-11</v>
@@ -1514,11 +1026,11 @@
         <v>1400</v>
       </c>
       <c r="N18">
-        <f>C18-D18*20-E18*0.8-F18*0.6-H18*5+I18*10+J18/300</f>
-        <v>24.8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>24.4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1537,7 +1049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1556,18 +1068,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C21" s="1">
         <f t="shared" ref="C21:M21" si="1">C3+C6</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D21" s="1">
         <f t="shared" si="1"/>
-        <v>0.34</v>
+        <v>0.4</v>
       </c>
       <c r="E21" s="1">
         <f t="shared" si="1"/>
@@ -1606,22 +1118,22 @@
         <v>0</v>
       </c>
       <c r="N21">
-        <f>C21-D21*20-E21*0.8-F21*0.6-H21*5+I21*10+J21/300</f>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>19.8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C22" s="1">
         <f t="shared" ref="C22:M22" si="2">C4+C5</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D22" s="1">
         <f t="shared" si="2"/>
-        <v>0.30000000000000004</v>
+        <v>0.44</v>
       </c>
       <c r="E22" s="1">
         <f t="shared" si="2"/>
@@ -1629,7 +1141,7 @@
       </c>
       <c r="F22" s="1">
         <f t="shared" si="2"/>
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G22" s="1">
         <f t="shared" si="2"/>
@@ -1660,22 +1172,22 @@
         <v>0</v>
       </c>
       <c r="N22">
-        <f>C22-D22*20-E22*0.8-F22*0.6-H22*5+I22*10+J22/300</f>
-        <v>19.600000000000001</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>19.399999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C23" s="1">
-        <f>C3+C7+C15+C16+C17</f>
+        <f t="shared" ref="C23:M23" si="3">C3+C7+C15+C16+C17</f>
         <v>15</v>
       </c>
       <c r="D23" s="1">
-        <f t="shared" ref="D23:M23" si="3">D3+D7+D15+D16+D17</f>
-        <v>0.44999999999999996</v>
+        <f t="shared" si="3"/>
+        <v>0.45999999999999996</v>
       </c>
       <c r="E23" s="1">
         <f t="shared" si="3"/>
@@ -1714,173 +1226,173 @@
         <v>2000</v>
       </c>
       <c r="N23">
-        <f t="shared" ref="N23:N29" si="4">C23-D23*20-E23*0.8-F23*0.6-H23*5+I23*10+J23/300</f>
-        <v>19.600000000000001</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>19.400000000000002</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C24" s="1">
-        <f>C3+C12+C11+C10</f>
-        <v>21</v>
+        <f t="shared" ref="C24:M24" si="4">C3+C12+C11+C10</f>
+        <v>20</v>
       </c>
       <c r="D24" s="1">
-        <f>D3+D12+D11+D10</f>
-        <v>0.49000000000000005</v>
+        <f t="shared" si="4"/>
+        <v>0.59999999999999987</v>
       </c>
       <c r="E24" s="1">
-        <f t="shared" ref="E24:M24" si="5">E3+E12+E11+E10</f>
+        <f t="shared" si="4"/>
         <v>-4</v>
       </c>
       <c r="F24" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>-6</v>
       </c>
       <c r="G24" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H24" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>-0.05</v>
       </c>
       <c r="I24" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J24" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K24" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L24" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="M24" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="N24">
-        <f t="shared" si="4"/>
-        <v>18.25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>15.050000000000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C25" s="1">
-        <f>C9+C13+C14</f>
-        <v>8</v>
+        <f t="shared" ref="C25:M25" si="5">C9+C13+C14</f>
+        <v>12</v>
       </c>
       <c r="D25" s="1">
-        <f t="shared" ref="D25:M25" si="6">D9+D13+D14</f>
-        <v>0.31</v>
+        <f t="shared" si="5"/>
+        <v>0.37999999999999995</v>
       </c>
       <c r="E25" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-10</v>
       </c>
       <c r="F25" s="1">
-        <f t="shared" si="6"/>
-        <v>-18</v>
+        <f t="shared" si="5"/>
+        <v>-15</v>
       </c>
       <c r="G25" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H25" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="I25" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J25" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="K25" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L25" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="M25" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1000</v>
       </c>
       <c r="N25">
-        <f t="shared" si="4"/>
-        <v>20.6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>21.400000000000002</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C26" s="1">
-        <f t="shared" ref="C26:M26" si="7">C3+C8+C18</f>
-        <v>16</v>
+        <f t="shared" ref="C26:M26" si="6">C3+C8+C18</f>
+        <v>15</v>
       </c>
       <c r="D26" s="1">
-        <f t="shared" si="7"/>
-        <v>0.5</v>
+        <f t="shared" si="6"/>
+        <v>0.53</v>
       </c>
       <c r="E26" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
+        <v>-11</v>
+      </c>
+      <c r="F26" s="1">
+        <f t="shared" si="6"/>
         <v>-10</v>
       </c>
-      <c r="F26" s="1">
-        <f t="shared" si="7"/>
-        <v>-9</v>
-      </c>
       <c r="G26" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H26" s="1">
-        <f t="shared" si="7"/>
-        <v>0.1</v>
+        <f t="shared" si="6"/>
+        <v>0</v>
       </c>
       <c r="I26" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J26" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="K26" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L26" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="M26" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>2600</v>
       </c>
       <c r="N26">
-        <f t="shared" si="4"/>
-        <v>18.899999999999999</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>19.2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1895,11 +1407,11 @@
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
       <c r="N27">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1914,11 +1426,11 @@
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
       <c r="N28">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1933,11 +1445,11 @@
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
       <c r="N29">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1952,11 +1464,11 @@
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
       <c r="N30">
-        <f t="shared" ref="N30:N31" si="8">C30-D30*20-E30*0.8-F30*0.6-H30*5+I30*10+J30/300</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1971,11 +1483,11 @@
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
       <c r="N31">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1994,7 +1506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2013,7 +1525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -2032,7 +1544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -2051,7 +1563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -2070,7 +1582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -2085,11 +1597,11 @@
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
       <c r="N37">
-        <f>C37-D37*20-E37*0.8-F37*0.6-H37*5+I37*10+J37/300</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2104,11 +1616,11 @@
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
       <c r="N38">
-        <f>C38-D38*20-E38*0.8-F38*0.6-H38*5+I38*10+J38/300</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2123,12 +1635,12 @@
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
       <c r="N39">
-        <f>C39-D39*20-E39*0.8-F39*0.6-H39*5+I39*10+J39/300</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>